<commit_message>
test: add formula and scale qualification evidence
</commit_message>
<xml_diff>
--- a/demo/workbooks/case_2_spreadsheet_control_failures.xlsx
+++ b/demo/workbooks/case_2_spreadsheet_control_failures.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="136">
   <si>
     <t xml:space="preserve">Case 2 — Spreadsheet control failures</t>
   </si>
@@ -420,9 +420,6 @@
   </si>
   <si>
     <t xml:space="preserve">Control line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expected signal</t>
   </si>
   <si>
     <t xml:space="preserve">Circular control A</t>
@@ -453,6 +450,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -764,192 +762,196 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="8" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="8" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="8" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="8" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="8" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="8" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="8" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="8" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="11" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="11" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="11" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="8" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="8" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="10" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="10" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="11" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="11" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="11" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="11" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="10" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="10" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="12" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="11" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="11" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="11" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="11" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="11" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="11" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1203,363 +1205,363 @@
   <dimension ref="A1:F25"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="10" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="10" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="10" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="11" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="12" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="13" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="13" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="13" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="F24" s="13" t="s">
+      <c r="F24" s="14" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="F25" s="13" t="s">
+      <c r="F25" s="14" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1590,301 +1592,301 @@
   <dimension ref="A1:F25"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="15" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="8" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="16" t="n">
         <v>10000000</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="17" t="n">
         <v>1800000</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="17" t="n">
         <v>650000</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="17" t="n">
         <v>125000</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="18" t="n">
         <v>0.05</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="8" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="30" t="s">
+      <c r="B25" s="31" t="s">
         <v>95</v>
       </c>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="30"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1918,124 +1920,124 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="15" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B7" s="31" t="n">
+      <c r="B7" s="32" t="n">
         <v>0.02</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="18" t="n">
         <v>0.04</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="18" t="n">
         <v>0.07</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2063,324 +2065,324 @@
   <dimension ref="A1:F25"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="15" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="11" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="B7" s="33" t="n">
+      <c r="B7" s="34" t="n">
         <f aca="false">Assumptions!B7*1.075</f>
         <v>10750000</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="D7" s="33" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="34" t="n">
+      <c r="B8" s="35" t="n">
         <f aca="false">Assumptions!B8</f>
         <v>1800000</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B9" s="34" t="n">
+      <c r="B9" s="35" t="n">
         <f aca="false">Assumptions!B9</f>
         <v>650000</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="36" t="n">
+      <c r="B10" s="37" t="n">
         <f aca="false">Assumptions!B10</f>
         <v>125000</v>
       </c>
-      <c r="C10" s="35" t="s">
+      <c r="C10" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="D10" s="35" t="s">
+      <c r="D10" s="36" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="34" t="n">
+      <c r="B11" s="35" t="n">
         <f aca="false">B8*Assumptions!B11</f>
         <v>90000</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="38" t="s">
         <v>119</v>
       </c>
-      <c r="B12" s="38" t="n">
+      <c r="B12" s="39" t="n">
         <f aca="false">SUM(B8:B9,B11)</f>
         <v>2540000</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="D12" s="37" t="s">
+      <c r="D12" s="38" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="B13" s="38" t="n">
-        <f aca="false">VLOOKUP(Assumptions!B12,'Lookup Table'!A7:B9,Assumptions!B13,FALSE())*B12</f>
+      <c r="B13" s="39" t="n">
+        <f aca="false">VLOOKUP(Assumptions!B12,'Lookup Table'!A7:B9,Assumptions!B13,TRUE())*B12</f>
         <v>101600</v>
       </c>
-      <c r="C13" s="37" t="s">
+      <c r="C13" s="38" t="s">
         <v>123</v>
       </c>
-      <c r="D13" s="37" t="s">
+      <c r="D13" s="38" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="39" t="s">
+      <c r="A14" s="40" t="s">
         <v>125</v>
       </c>
-      <c r="B14" s="40" t="n">
+      <c r="B14" s="41" t="n">
         <f aca="false">SUM(B12:B13)</f>
         <v>2641600</v>
       </c>
-      <c r="C14" s="41" t="s">
+      <c r="C14" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="D14" s="42" t="s">
+      <c r="D14" s="43" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="8" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="30" t="s">
+      <c r="B25" s="31" t="s">
         <v>95</v>
       </c>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="30"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -2414,129 +2416,135 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>128</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="E3" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="F3" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="F3" s="14" t="s">
-        <v>129</v>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C4" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="C5" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="D5" s="43" t="s">
-        <v>130</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="n">
+        <f aca="false">SUM(C1:C2,C4:C5)</f>
+        <v>4</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="45" t="s">
         <v>132</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="44" t="s">
-        <v>133</v>
-      </c>
-      <c r="B7" s="45" t="e">
+      <c r="B7" s="46" t="e">
         <f aca="false">'Circular Control'!B8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="44" t="s">
+      <c r="D7" s="45" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="36" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="B8" s="46" t="e">
+      <c r="B8" s="47" t="e">
         <f aca="false">'Circular Control'!B7</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C8" s="35" t="s">
+      <c r="C8" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="35" t="s">
-        <v>136</v>
+      <c r="D8" s="36" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>